<commit_message>
More fixes and changes
</commit_message>
<xml_diff>
--- a/resources/data-imports/World Gems/location-gems.xlsx
+++ b/resources/data-imports/World Gems/location-gems.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI29"/>
+  <dimension ref="A1:AJ26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <sheetData>
     <row r="1">
@@ -592,6 +592,11 @@
           <t>monster_atonement_range</t>
         </is>
       </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>gem_world_name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -616,122 +621,127 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.001-0.005</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Hollow Beneath the Stone</t>
         </is>
       </c>
     </row>
@@ -758,122 +768,127 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>0.02-0.08</t>
+          <t>0.002-0.008</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Halls That Remember Nothing</t>
         </is>
       </c>
     </row>
@@ -900,122 +915,127 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>0.04-0.16</t>
+          <t>0.004-0.016</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Rotting Crown of the Deep</t>
         </is>
       </c>
     </row>
@@ -1042,117 +1062,122 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Bones of the Drowned Tide</t>
         </is>
       </c>
     </row>
@@ -1179,117 +1204,122 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.01-0.025</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0189-0.02625</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Bound in Endless Malice</t>
         </is>
       </c>
     </row>
@@ -1316,137 +1346,142 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>Harbor of Severed Oaths</t>
         </is>
       </c>
     </row>
@@ -1473,137 +1508,142 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Silent Congregation's Vigil</t>
         </is>
       </c>
     </row>
@@ -1630,137 +1670,142 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>Ruin of Green Embers</t>
         </is>
       </c>
     </row>
@@ -1787,137 +1832,142 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>Vault of Unmourned Names</t>
         </is>
       </c>
     </row>
@@ -1944,137 +1994,142 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>0.18-0.35</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>Where the Soil Refuses Rest</t>
         </is>
       </c>
     </row>
@@ -2101,117 +2156,122 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>Ashes of the Last Hearth</t>
         </is>
       </c>
     </row>
@@ -2238,117 +2298,122 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>Fields That Scream at Dawn</t>
         </is>
       </c>
     </row>
@@ -2375,117 +2440,122 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>Crimson Drift of Bone</t>
         </is>
       </c>
     </row>
@@ -2512,117 +2582,122 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI15" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>No Map Remembers This Path</t>
         </is>
       </c>
     </row>
@@ -2649,117 +2724,122 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>Paws Beneath the Frost</t>
         </is>
       </c>
     </row>
@@ -2786,117 +2866,122 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>Coffers Beneath the Ice</t>
         </is>
       </c>
     </row>
@@ -2923,117 +3008,122 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>Hull of the Forgotten Cold</t>
         </is>
       </c>
     </row>
@@ -3060,117 +3150,122 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI19" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>The Bloodied Prayer</t>
         </is>
       </c>
     </row>
@@ -3197,117 +3292,122 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI20" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ20" t="inlineStr">
+        <is>
+          <t>Tunnels of Golden Lies</t>
         </is>
       </c>
     </row>
@@ -3334,1278 +3434,892 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>0.22-0.50</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI21" t="inlineStr">
         <is>
-          <t>0.504-0.6825</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ21" t="inlineStr">
+        <is>
+          <t>Hush of the Occupation</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>Underwater Caves Gem Profile</t>
+          <t>Gold Mine Gem Profile</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Location gem profile for Underwater Caves on Surface, raised five percent above its plane baseline.</t>
+          <t>Location gem profile for Gold Mine on Shadow Plane, raised five percent above its plane baseline.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Surface</t>
+          <t>Shadow Plane</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Underwater Caves</t>
+          <t>Gold Mine</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>0.01-0.05</t>
+          <t>0.008-0.02</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
         </is>
       </c>
       <c r="AI22" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0063-0.0126</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>A Vein That Bites Back</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gold Mine Gem Profile</t>
+          <t>Purgatories Dungeons Gem Profile</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Location gem profile for Gold Mine on Shadow Plane, raised five percent above its plane baseline.</t>
+          <t>Location gem profile for Purgatories Dungeons on Purgatory, raised five percent above its plane baseline.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Shadow Plane</t>
+          <t>Purgatory</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Gold Mine</t>
+          <t>Purgatories Dungeons</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>0.08-0.20</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI23" t="inlineStr">
         <is>
-          <t>0.063-0.126</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>Cells of the Unforgiven</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tear in the Fabric of Time Gem Profile</t>
+          <t>Purgatory Smiths House Gem Profile</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Location gem profile for Tear in the Fabric of Time on Hell, raised five percent above its plane baseline.</t>
+          <t>Location gem profile for Purgatory Smiths House on Purgatory, raised five percent above its plane baseline.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Hell</t>
+          <t>Purgatory</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Tear in the Fabric of Time</t>
+          <t>Purgatory Smiths House</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.015-0.03</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI24" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>Forge of Broken Children</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>Twisted Dimensional Gate Gem Profile</t>
+          <t>Cave of Shadows Gem Profile</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Location gem profile for Twisted Dimensional Gate on Hell, raised five percent above its plane baseline.</t>
+          <t>Location gem profile for Cave of Shadows on Twisted Memories, raised five percent above its plane baseline.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hell</t>
+          <t>Twisted Memories</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Twisted Dimensional Gate</t>
+          <t>Cave of Shadows</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>0.10-0.25</t>
+          <t>0.018-0.035</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">
         <is>
-          <t>0.189-0.2625</t>
+          <t>0.0504-0.06825</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>The Devouring Dark</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>Purgatories Dungeons Gem Profile</t>
+          <t>The Old Church Gem Profile</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Location gem profile for Purgatories Dungeons on Purgatory, raised five percent above its plane baseline.</t>
+          <t>Location gem profile for The Old Church on The Ice Plane, raised five percent above its plane baseline.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Purgatory</t>
+          <t>The Ice Plane</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Purgatories Dungeons</t>
+          <t>The Old Church</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>0.15-0.30</t>
+          <t>0.022-0.05</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AB26" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AC26" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AD26" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
         </is>
       </c>
       <c r="AI26" t="inlineStr">
         <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Purgatory Smiths House Gem Profile</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Location gem profile for Purgatory Smiths House on Purgatory, raised five percent above its plane baseline.</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Purgatory</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Purgatory Smiths House</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>0.15-0.30</t>
-        </is>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AB27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AC27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AD27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AE27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AF27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AG27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AI27" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Cave of Shadows Gem Profile</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Location gem profile for Cave of Shadows on Twisted Memories, raised five percent above its plane baseline.</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Twisted Memories</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Cave of Shadows</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>0.18-0.35</t>
-        </is>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="Z28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AB28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AC28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AD28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AE28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AF28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AG28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-      <c r="AI28" t="inlineStr">
-        <is>
-          <t>0.504-0.6825</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>The Old Church Gem Profile</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Location gem profile for The Old Church on The Ice Plane, raised five percent above its plane baseline.</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>The Ice Plane</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>The Old Church</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>0.22-0.50</t>
-        </is>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="W29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="Z29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AE29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AF29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AG29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
-        </is>
-      </c>
-      <c r="AI29" t="inlineStr">
-        <is>
-          <t>0.315-0.5775</t>
+          <t>0.0315-0.05775</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>Sanctuary of Rotten Hymns</t>
         </is>
       </c>
     </row>

</xml_diff>